<commit_message>
Add data I 2026
</commit_message>
<xml_diff>
--- a/df_followers.xlsx
+++ b/df_followers.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lapto\OneDrive\Pulpit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lapto\OneDrive\Pulpit\Scraper Social Media\Social Media Scraper 2025\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7546D8-A490-40DF-B560-F7FBAF42B68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E11001F-DE43-4048-A2BF-4139222B228D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
+    <t>Pismo</t>
+  </si>
+  <si>
     <t>Facebook</t>
   </si>
   <si>
@@ -40,6 +43,9 @@
     <t>X</t>
   </si>
   <si>
+    <t xml:space="preserve">YouTube </t>
+  </si>
+  <si>
     <t>Suma</t>
   </si>
   <si>
@@ -353,12 +359,6 @@
   </si>
   <si>
     <t>Olivia</t>
-  </si>
-  <si>
-    <t>Tytuł</t>
-  </si>
-  <si>
-    <t>YouTube</t>
   </si>
 </sst>
 </file>
@@ -737,36 +737,36 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2">
         <v>768000</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2">
         <v>1500000</v>
@@ -824,7 +824,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>824000</v>
@@ -853,7 +853,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2">
         <v>957000</v>
@@ -882,7 +882,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2">
         <v>524000</v>
@@ -911,7 +911,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" s="2">
         <v>532000</v>
@@ -940,7 +940,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2">
         <v>196000</v>
@@ -969,7 +969,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2">
         <v>516000</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" s="2">
         <v>212000</v>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" s="2">
         <v>596000</v>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B12" s="2">
         <v>312000</v>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B13" s="2">
         <v>330000</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2">
         <v>290000</v>
@@ -1143,7 +1143,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B15" s="2">
         <v>328000</v>
@@ -1172,7 +1172,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B16" s="2">
         <v>226000</v>
@@ -1201,7 +1201,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B17" s="2">
         <v>358000</v>
@@ -1230,7 +1230,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B18" s="2">
         <v>131000</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B19" s="2">
         <v>43000</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B20" s="2">
         <v>329000</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B21" s="2">
         <v>157000</v>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B22" s="2">
         <v>254000</v>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B23" s="2">
         <v>124000</v>
@@ -1404,7 +1404,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B24" s="2">
         <v>250000</v>
@@ -1433,7 +1433,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B25" s="2">
         <v>113000</v>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B26" s="2">
         <v>200000</v>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B27" s="2">
         <v>157000</v>
@@ -1520,7 +1520,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B28" s="2">
         <v>194000</v>
@@ -1549,7 +1549,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B29" s="2">
         <v>189000</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B30" s="2">
         <v>192000</v>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B31" s="2">
         <v>189000</v>
@@ -1636,7 +1636,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B32" s="2">
         <v>177000</v>
@@ -1665,7 +1665,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B33" s="2">
         <v>162000</v>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B34" s="2">
         <v>136000</v>
@@ -1723,7 +1723,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B35" s="2">
         <v>153000</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B36" s="2">
         <v>151000</v>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B37" s="2">
         <v>65000</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B38" s="2">
         <v>157000</v>
@@ -1839,7 +1839,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B39" s="2">
         <v>24000</v>
@@ -1868,7 +1868,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B40" s="2">
         <v>125000</v>
@@ -1897,7 +1897,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B41" s="2">
         <v>145000</v>
@@ -1926,7 +1926,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B42" s="2">
         <v>102000</v>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B43" s="2">
         <v>49000</v>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B44" s="2">
         <v>105000</v>
@@ -2013,7 +2013,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B45" s="2">
         <v>39000</v>
@@ -2042,7 +2042,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B46" s="2">
         <v>102000</v>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B47" s="2">
         <v>44000</v>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B48" s="2">
         <v>89000</v>
@@ -2129,7 +2129,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B49" s="2">
         <v>80000</v>
@@ -2158,7 +2158,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B50" s="2">
         <v>80000</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B51" s="2">
         <v>82000</v>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B52" s="2">
         <v>79000</v>
@@ -2245,7 +2245,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B53" s="2">
         <v>80000</v>
@@ -2274,7 +2274,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B54" s="2">
         <v>37000</v>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B55" s="2">
         <v>35000</v>
@@ -2332,7 +2332,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B56" s="2">
         <v>54000</v>
@@ -2361,7 +2361,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B57" s="2">
         <v>22000</v>
@@ -2390,7 +2390,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B58" s="2">
         <v>52000</v>
@@ -2419,7 +2419,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B59" s="2">
         <v>45000</v>
@@ -2448,7 +2448,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B60" s="2">
         <v>37000</v>
@@ -2477,7 +2477,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B61" s="2">
         <v>43000</v>
@@ -2506,7 +2506,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B62" s="2">
         <v>39000</v>
@@ -2535,7 +2535,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B63" s="2">
         <v>40000</v>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B64" s="2">
         <v>35000</v>
@@ -2593,7 +2593,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B65" s="2">
         <v>37000</v>
@@ -2622,7 +2622,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B66" s="2">
         <v>32000</v>
@@ -2651,7 +2651,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B67" s="2">
         <v>35000</v>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B68" s="2">
         <v>22000</v>
@@ -2709,7 +2709,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B69" s="2">
         <v>31000</v>
@@ -2738,7 +2738,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B70" s="2">
         <v>26000</v>
@@ -2767,7 +2767,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B71" s="2">
         <v>28000</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B72" s="2">
         <v>31000</v>
@@ -2825,7 +2825,7 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B73" s="2">
         <v>28000</v>
@@ -2854,7 +2854,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B74" s="2">
         <v>28000</v>
@@ -2883,7 +2883,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B75" s="2">
         <v>25000</v>
@@ -2912,7 +2912,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B76" s="2">
         <v>26000</v>
@@ -2941,7 +2941,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B77" s="2">
         <v>25000</v>
@@ -2970,7 +2970,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B78" s="2">
         <v>22000</v>
@@ -2999,7 +2999,7 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B79" s="2">
         <v>22000</v>
@@ -3028,7 +3028,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B80" s="2">
         <v>15000</v>
@@ -3057,7 +3057,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B81" s="2">
         <v>0</v>
@@ -3086,7 +3086,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B82" s="2">
         <v>8100</v>
@@ -3115,7 +3115,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B83" s="2">
         <v>9800</v>
@@ -3144,7 +3144,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B84" s="2">
         <v>3000</v>
@@ -3173,7 +3173,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B85" s="2">
         <v>4200</v>
@@ -3202,7 +3202,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B86" s="2">
         <v>9700</v>
@@ -3231,7 +3231,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B87" s="2">
         <v>9800</v>
@@ -3260,7 +3260,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B88" s="2">
         <v>6900</v>
@@ -3289,7 +3289,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B89" s="2">
         <v>8000</v>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B90" s="2">
         <v>7800</v>
@@ -3347,7 +3347,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B91" s="2">
         <v>7000</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B92" s="2">
         <v>6300</v>
@@ -3405,7 +3405,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B93" s="2">
         <v>0</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B94" s="2">
         <v>5900</v>
@@ -3463,7 +3463,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B95" s="2">
         <v>5800</v>
@@ -3492,7 +3492,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B96" s="2">
         <v>1400</v>
@@ -3521,7 +3521,7 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B97" s="2">
         <v>3500</v>
@@ -3550,7 +3550,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B98" s="2">
         <v>2100</v>
@@ -3579,7 +3579,7 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B99" s="2">
         <v>2400</v>
@@ -3608,7 +3608,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B100" s="2">
         <v>2500</v>
@@ -3637,7 +3637,7 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B101" s="2">
         <v>2300</v>
@@ -3666,7 +3666,7 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B102" s="2">
         <v>2200</v>
@@ -3695,7 +3695,7 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B103" s="2">
         <v>2100</v>
@@ -3724,7 +3724,7 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B104" s="2">
         <v>1500</v>
@@ -3753,7 +3753,7 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B105" s="2">
         <v>1000</v>

</xml_diff>